<commit_message>
add locked_out_user test case to login and testsheet.xlsx updated
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="18">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -74,6 +74,23 @@
 2. get the url of the page loaded.
 3. get the title from the url.
 4. check if the swag labs present or not in the title for test is "pass" or "fail". </t>
+  </si>
+  <si>
+    <t>TC_003</t>
+  </si>
+  <si>
+    <t>lockedout_user_login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To test the functionality of login of locked out users
+(username = locked_out_user, password = secret_sauce) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open  the url of the saucedemo webpage. 
+2. put the credentials as (username = locked_out_user , password = secret_sauce).
+3. click on login button.
+4. get the text of the error message . 
+4. check if the error message contains locked out then it is "pass " otherwise "fail". </t>
   </si>
 </sst>
 </file>
@@ -461,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -520,6 +537,23 @@
       </c>
       <c r="E3" s="7" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="112.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added the problem_user login and testsheet updated
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10656" windowHeight="4380"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10656" windowHeight="6516"/>
   </bookViews>
   <sheets>
     <sheet name="GOVIND" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="22">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -91,6 +91,23 @@
 3. click on login button.
 4. get the text of the error message . 
 4. check if the error message contains locked out then it is "pass " otherwise "fail". </t>
+  </si>
+  <si>
+    <t>TC_004</t>
+  </si>
+  <si>
+    <t>problem_user_login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To test the functionality of login of problrm users
+(username = problem_user, password = secret_sauce) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open  the url of the saucedemo webpage. 
+2. put the credentials as (username = problem_user , password = secret_sauce).
+3. click on login button.
+4. get the link of the new webpage after login as actualurl. 
+4. check if the actualurl contains inventory.html then it is "pass - Problem User Login Successful" otherwise "fail  - Problem User Login Failed". </t>
   </si>
 </sst>
 </file>
@@ -478,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -554,6 +571,23 @@
       </c>
       <c r="E4" s="7" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added the performance_glitch_user login test case and testsheet updated with it
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10656" windowHeight="6516"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13008" windowHeight="5796"/>
   </bookViews>
   <sheets>
     <sheet name="GOVIND" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
     <sheet name="ASHUTOSH" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
+  <oleSize ref="E5:K6"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="26">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -99,15 +99,33 @@
     <t>problem_user_login</t>
   </si>
   <si>
-    <t xml:space="preserve">To test the functionality of login of problrm users
-(username = problem_user, password = secret_sauce) </t>
-  </si>
-  <si>
     <t xml:space="preserve">1. open  the url of the saucedemo webpage. 
 2. put the credentials as (username = problem_user , password = secret_sauce).
 3. click on login button.
 4. get the link of the new webpage after login as actualurl. 
 4. check if the actualurl contains inventory.html then it is "pass - Problem User Login Successful" otherwise "fail  - Problem User Login Failed". </t>
+  </si>
+  <si>
+    <t>TC_005</t>
+  </si>
+  <si>
+    <t>performance_glitch_user_login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To test the functionality of login of problem users
+(username = problem_user, password = secret_sauce) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">To test the functionality of login of performance_glitch users
+(username = performance_glitch_user,
+ password = secret_sauce) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open  the url of the saucedemo webpage. 
+2. put the credentials as (username = performance_glitch_user , password = secret_sauce).
+3. click on login button.
+4. get the link of the new webpage after login as actualurl. 
+4. check if the actualurl contains inventory.html then it is "pass - performance glitch user Login Successful" otherwise "fail  - performance glitch user Login Failed". </t>
   </si>
 </sst>
 </file>
@@ -495,12 +513,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="16.5546875" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.21875" customWidth="1"/>
     <col min="4" max="4" width="56.21875" customWidth="1"/>
     <col min="5" max="5" width="44.33203125" customWidth="1"/>
   </cols>
@@ -584,10 +602,27 @@
         <v>19</v>
       </c>
       <c r="D5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="7" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="148.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>21</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added error_user and visual_user login and updated testsheet
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -3,6 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="164011"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\eclipse-workspace\SauceDemo\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="13008" windowHeight="5796"/>
   </bookViews>
@@ -14,7 +19,6 @@
     <sheet name="ASHUTOSH" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="E5:K6"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="34">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -99,33 +103,67 @@
     <t>problem_user_login</t>
   </si>
   <si>
-    <t xml:space="preserve">1. open  the url of the saucedemo webpage. 
+    <t>TC_005</t>
+  </si>
+  <si>
+    <t>performance_glitch_user_login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To test the functionality of login of problem users
+(username = problem_user, password = secret_sauce) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">To test the functionality of login of performance_glitch users
+(username = performance_glitch_user,
+ password = secret_sauce) </t>
+  </si>
+  <si>
+    <t>TC_006</t>
+  </si>
+  <si>
+    <t>TC_007</t>
+  </si>
+  <si>
+    <t>error_user_login</t>
+  </si>
+  <si>
+    <t>visual_user_login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To test the functionality of login of error users
+(username = error_user,password = secret_sauce) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">To test the functionality of login of visual users
+(username =visual_user,password = secret_sauce) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
 2. put the credentials as (username = problem_user , password = secret_sauce).
 3. click on login button.
 4. get the link of the new webpage after login as actualurl. 
 4. check if the actualurl contains inventory.html then it is "pass - Problem User Login Successful" otherwise "fail  - Problem User Login Failed". </t>
   </si>
   <si>
-    <t>TC_005</t>
-  </si>
-  <si>
-    <t>performance_glitch_user_login</t>
-  </si>
-  <si>
-    <t xml:space="preserve">To test the functionality of login of problem users
-(username = problem_user, password = secret_sauce) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">To test the functionality of login of performance_glitch users
-(username = performance_glitch_user,
- password = secret_sauce) </t>
-  </si>
-  <si>
     <t xml:space="preserve">1. open  the url of the saucedemo webpage. 
+2. put the credentials as (username = visual_user , password = secret_sauce).
+3. click on login button.
+4. get the link of the new webpage after login as actualurl. 
+4. check if the actualurl contains inventory.html then it is "pass - performance glitch user Login Successful" otherwise "fail  - performance glitch user Login Failed". </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open  the url of the saucedemo webpage. 
+2. put the credentials as (username = error_user , password = secret_sauce).
+3. click on login button.
+4. get the link of the new webpage after login as actualurl. 
+4. check if the actualurl contains inventory.html then it is "PASS" otherwise "Fail ". </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
 2. put the credentials as (username = performance_glitch_user , password = secret_sauce).
 3. click on login button.
 4. get the link of the new webpage after login as actualurl. 
-4. check if the actualurl contains inventory.html then it is "pass - performance glitch user Login Successful" otherwise "fail  - performance glitch user Login Failed". </t>
+4. check if the actualurl contains inventory.html then it is "PASS" otherwise "Fail". </t>
   </si>
 </sst>
 </file>
@@ -513,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -602,27 +640,61 @@
         <v>19</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="148.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="178.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="D6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="190.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="C7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>25</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added test-case that removes items from cart
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="8400" activeTab="1"/>
+    <workbookView windowWidth="12420" windowHeight="9000" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="GOVIND" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="31">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -112,7 +112,9 @@
     <t>Verify Product in Cart</t>
   </si>
   <si>
-    <t>Validate that the selected product is correctly displayed in the cart</t>
+    <t>Validate that the selected 
+product is correctly 
+displayed in the cart</t>
   </si>
   <si>
     <t>1. Open SauceDemo website. 
@@ -132,7 +134,7 @@
   </si>
   <si>
     <t>Validate that the selected product is
- correctly displayed in the cart</t>
+correctly displayed in the cart</t>
   </si>
   <si>
     <t>1. Open SauceDemo website.
@@ -142,6 +144,27 @@
 5. Click Add to cart. 
 6. Open the cart. 
 7. Check the product name and price. 8. Verify that the product name is Sauce Labs Backpack and the price is $29.99.</t>
+  </si>
+  <si>
+    <t>TC_CART_005</t>
+  </si>
+  <si>
+    <t>Remove Product from Cart</t>
+  </si>
+  <si>
+    <t>To check whether the user 
+can remove a product 
+from the cart</t>
+  </si>
+  <si>
+    <t>1. Open the SauceDemo website.
+2. Enter valid username and password.
+3. Click Login.
+4. Select Sauce Labs Backpack.
+5. Click Add to cart.
+6. Open the cart.
+7. Click Remove for Sauce Labs Backpack.
+8. Verify that the product is removed from the cart.</t>
   </si>
 </sst>
 </file>
@@ -760,7 +783,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="29"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="35"/>
@@ -771,6 +794,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="41" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1109,53 +1141,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" ht="102.6" customHeight="1" spans="1:5">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="12" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" ht="93.6" customHeight="1" spans="1:5">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="12" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1169,12 +1201,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="4"/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="17.5555555555556" customWidth="1"/>
     <col min="2" max="2" width="16.5555555555556" customWidth="1"/>
-    <col min="3" max="3" width="18.4444444444444" customWidth="1"/>
+    <col min="3" max="3" width="25.1111111111111" customWidth="1"/>
     <col min="4" max="4" width="25.3333333333333" customWidth="1"/>
     <col min="5" max="5" width="33.2222222222222" customWidth="1"/>
   </cols>
@@ -1223,7 +1255,7 @@
       <c r="C3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E3" s="6" t="s">
@@ -1245,6 +1277,23 @@
       </c>
       <c r="E4" s="6" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="5" ht="144" spans="1:5">
+      <c r="A5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
some change in TC_008 and added a new test case as nousername_withpassword as TC_009 and update the testsheet also
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="59">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -209,13 +209,6 @@
   </si>
   <si>
     <t xml:space="preserve">1. open the url of the saucedemo webpage. 
-2. put the credentials as (username = any username that mention).
-3. click on login button.
-4. get the error as Epic sadface: Username is required. 
-5. if error present then it is "PASSED" otherwise "FAILED". </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
 2. put the credentials as (username = performance_glitch_user , password = secret_sauce).
 3. click on login button.
 4. get the link of the new webpage after login as actualurl. 
@@ -256,17 +249,47 @@
 4. get the link of the new webpage after login as actualurl. 
 5. check if the actualurl contains inventory.html then it is "PASS" otherwise "Fail ". </t>
   </si>
+  <si>
+    <t>TC_009</t>
+  </si>
+  <si>
+    <t>nousername_withpassword</t>
+  </si>
+  <si>
+    <t>To test the functionality of login of user with no username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
+2. put the credentials as (username = any username that mention).
+3. click on login button.
+4. get the error as Epic sadface: Password is required. 
+5. if error present then it is "PASSED" otherwise "FAILED". </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
+2. put the credentials as (password = secret_sauce that mention).
+3. click on login button.
+4. get the error as Epic sadface: Username is required. 
+5. if error present then it is "PASSED" otherwise "FAILED". </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -389,24 +412,24 @@
   </borders>
   <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -422,20 +445,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -724,7 +756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -734,7 +766,7 @@
     <col min="5" max="5" width="44.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -751,7 +783,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="102.6" customHeight="1">
+    <row r="2" spans="1:6" ht="102.6" customHeight="1">
       <c r="A2" s="11" t="s">
         <v>5</v>
       </c>
@@ -768,7 +800,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="93.6" customHeight="1">
+    <row r="3" spans="1:6" ht="93.6" customHeight="1">
       <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
@@ -782,10 +814,10 @@
         <v>12</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="100.8">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="100.8">
       <c r="A4" s="13" t="s">
         <v>5</v>
       </c>
@@ -799,10 +831,10 @@
         <v>32</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="129.6">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="129.6">
       <c r="A5" s="13" t="s">
         <v>5</v>
       </c>
@@ -816,10 +848,10 @@
         <v>35</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="144">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="144">
       <c r="A6" s="13" t="s">
         <v>5</v>
       </c>
@@ -833,10 +865,10 @@
         <v>38</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="115.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="115.2">
       <c r="A7" s="13" t="s">
         <v>5</v>
       </c>
@@ -850,10 +882,10 @@
         <v>41</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="129.6">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="129.6">
       <c r="A8" s="15" t="s">
         <v>5</v>
       </c>
@@ -867,11 +899,11 @@
         <v>44</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="115.2">
-      <c r="A9" s="15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="115.2">
+      <c r="A9" s="16" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="13" t="s">
@@ -883,8 +915,26 @@
       <c r="D9" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="E9" s="14" t="s">
-        <v>48</v>
+      <c r="E9" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" s="18"/>
+    </row>
+    <row r="10" spans="1:6" ht="115.2">
+      <c r="A10" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated the testsheet with the tc_010(alphabetinput_to_username) and tc_011(numericinput_to_username)
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14520" windowHeight="5748"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14520" windowHeight="3936"/>
   </bookViews>
   <sheets>
     <sheet name="GOVIND" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="67">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -266,23 +266,58 @@
 5. if error present then it is "PASSED" otherwise "FAILED". </t>
   </si>
   <si>
+    <t>TC_010</t>
+  </si>
+  <si>
+    <t>TC_011</t>
+  </si>
+  <si>
+    <t>alphabetinput_to_username</t>
+  </si>
+  <si>
+    <t>numericinput_to_username</t>
+  </si>
+  <si>
     <t xml:space="preserve">1. open the url of the saucedemo webpage. 
-2. put the credentials as (password = secret_sauce that mention).
-3. click on login button.
-4. get the error as Epic sadface: Username is required. 
-5. if error present then it is "PASSED" otherwise "FAILED". </t>
+2. Enter the aplhabets in the username variable.
+4. if error present then it is "PASSED" otherwise "FAILED". </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
+2. enter the alphabet to the username variable.
+3. check that the entered data is entering in the username field.
+4. if entered then it is "PASSED: Alphabet keys work" otherwise "FAILED: Alphabet keys do not work". </t>
+  </si>
+  <si>
+    <t>To test the functionality of entering of the numeric values to the username field</t>
+  </si>
+  <si>
+    <t>To test the functionality of entering of the alphabets to the username field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
+2. enter the numeric value to the username variable.
+3. check that the entered data is entering in the username field.
+4. if entered then it is "PASSED: Number keys work" otherwise "FAILED: Number keys do not work". </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -412,24 +447,24 @@
   </borders>
   <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -445,30 +480,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="12">
@@ -756,7 +797,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -920,7 +961,7 @@
       </c>
       <c r="F9" s="18"/>
     </row>
-    <row r="10" spans="1:6" ht="115.2">
+    <row r="10" spans="1:6" ht="57.6">
       <c r="A10" s="16" t="s">
         <v>5</v>
       </c>
@@ -933,8 +974,42 @@
       <c r="D10" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="20" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="108" customHeight="1">
+      <c r="A11" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="13" t="s">
         <v>58</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="86.4">
+      <c r="A12" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add a new test case named as specialsymbol_input_to_username to LOGIN_FUNCTIONALITY and updated the testsheet accordingly
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14520" windowHeight="3936" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14520" windowHeight="3936"/>
   </bookViews>
   <sheets>
     <sheet name="GOVIND" sheetId="1" r:id="rId1"/>
@@ -14,12 +14,12 @@
     <sheet name="ASHUTOSH" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A5:G7"/>
+  <oleSize ref="B12:E18"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="94">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -413,17 +413,39 @@
 4. Open the cart page. 
 5. Verify that the product quantity is displayed as 1.</t>
   </si>
+  <si>
+    <t>TC_012</t>
+  </si>
+  <si>
+    <t>specialsymbolinput_to_username</t>
+  </si>
+  <si>
+    <t>To test the functionality of entering of the special symbols to the username field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
+2. enter the symbol to the username variable.
+3. check that the entered data is entering in the username field.
+4. if entered then it is "TEST CASE PASS" otherwise "TEST CASE FAIL". </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -560,24 +582,24 @@
   </borders>
   <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -590,30 +612,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -907,12 +935,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="16.5546875" customWidth="1"/>
-    <col min="3" max="3" width="27.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31" customWidth="1"/>
     <col min="4" max="4" width="56.21875" customWidth="1"/>
     <col min="5" max="5" width="44.33203125" customWidth="1"/>
   </cols>
@@ -1120,6 +1148,23 @@
       </c>
       <c r="E12" s="19" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="86.4">
+      <c r="A13" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added a new test case named as alphabetinput_to_password to LOGIN_FUNCTIONALITY and updated the testsheet accordingly
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="12276" windowHeight="9000" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14520" windowHeight="3936"/>
   </bookViews>
   <sheets>
     <sheet name="GOVIND" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,8 @@
     <sheet name="NITISH" sheetId="6" r:id="rId4"/>
     <sheet name="ASHUTOSH" sheetId="7" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A12:D13"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="102">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -463,18 +464,27 @@
 8. Verify that both products are 
 still displayed in the cart.</t>
   </si>
+  <si>
+    <t>TC_013</t>
+  </si>
+  <si>
+    <t>alphabetinput_to_password</t>
+  </si>
+  <si>
+    <t>To test the functionality of entering of the alphabets to the password field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
+2. enter the alphabet to the password variable.
+3. check that the entered data is entering in the password field.
+4. if entered then it is "PASSED: Alphabet keys work" otherwise "FAILED: Alphabet keys do not work". </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="24">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -505,150 +515,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
@@ -656,7 +522,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -671,13 +537,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -695,174 +561,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -870,254 +580,27 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="55">
+  <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="29"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="35"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="31"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="45"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1133,90 +616,57 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="41" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="54" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="54" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="54" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="54" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="54" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="55">
+  <cellStyles count="12">
+    <cellStyle name="40% - Accent2" xfId="2" builtinId="35"/>
+    <cellStyle name="40% - Accent2 2" xfId="6"/>
+    <cellStyle name="40% - Accent3" xfId="3" builtinId="39"/>
+    <cellStyle name="40% - Accent3 2" xfId="7"/>
+    <cellStyle name="Accent2" xfId="1" builtinId="33"/>
+    <cellStyle name="Accent2 2" xfId="8"/>
+    <cellStyle name="Accent5" xfId="4" builtinId="45"/>
+    <cellStyle name="Accent5 2" xfId="9"/>
+    <cellStyle name="Accent6" xfId="5" builtinId="49"/>
+    <cellStyle name="Accent6 2" xfId="10"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="40% - Accent2 2" xfId="49"/>
-    <cellStyle name="40% - Accent3 2" xfId="50"/>
-    <cellStyle name="Accent2 2" xfId="51"/>
-    <cellStyle name="Accent5 2" xfId="52"/>
-    <cellStyle name="Accent6 2" xfId="53"/>
-    <cellStyle name="Normal 2" xfId="54"/>
+    <cellStyle name="Normal 2" xfId="11"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1474,20 +924,20 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="16.5555555555556" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
     <col min="3" max="3" width="31" customWidth="1"/>
-    <col min="4" max="4" width="56.2222222222222" customWidth="1"/>
-    <col min="5" max="5" width="44.3333333333333" customWidth="1"/>
+    <col min="4" max="4" width="56.21875" customWidth="1"/>
+    <col min="5" max="5" width="44.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1507,7 +957,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" ht="102.6" customHeight="1" spans="1:6">
+    <row r="2" spans="1:6" ht="102.6" customHeight="1">
       <c r="A2" s="11" t="s">
         <v>5</v>
       </c>
@@ -1524,7 +974,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" ht="93.6" customHeight="1" spans="1:6">
+    <row r="3" spans="1:6" ht="93.6" customHeight="1">
       <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
@@ -1541,7 +991,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" ht="100.8" spans="1:6">
+    <row r="4" spans="1:6" ht="100.8">
       <c r="A4" s="13" t="s">
         <v>5</v>
       </c>
@@ -1558,7 +1008,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" ht="129.6" spans="1:6">
+    <row r="5" spans="1:6" ht="129.6">
       <c r="A5" s="13" t="s">
         <v>5</v>
       </c>
@@ -1575,7 +1025,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" ht="144" spans="1:6">
+    <row r="6" spans="1:6" ht="144">
       <c r="A6" s="13" t="s">
         <v>5</v>
       </c>
@@ -1592,7 +1042,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" ht="115.2" spans="1:6">
+    <row r="7" spans="1:6" ht="115.2">
       <c r="A7" s="13" t="s">
         <v>5</v>
       </c>
@@ -1609,7 +1059,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" ht="115.2" spans="1:6">
+    <row r="8" spans="1:6" ht="129.6">
       <c r="A8" s="15" t="s">
         <v>5</v>
       </c>
@@ -1626,7 +1076,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" ht="100.8" spans="1:6">
+    <row r="9" spans="1:6" ht="115.2">
       <c r="A9" s="15" t="s">
         <v>5</v>
       </c>
@@ -1644,7 +1094,7 @@
       </c>
       <c r="F9" s="17"/>
     </row>
-    <row r="10" ht="57.6" spans="1:6">
+    <row r="10" spans="1:6" ht="57.6">
       <c r="A10" s="15" t="s">
         <v>5</v>
       </c>
@@ -1661,7 +1111,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" ht="108" customHeight="1" spans="1:6">
+    <row r="11" spans="1:6" ht="108" customHeight="1">
       <c r="A11" s="15" t="s">
         <v>5</v>
       </c>
@@ -1671,14 +1121,14 @@
       <c r="C11" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="19" t="s">
         <v>44</v>
       </c>
       <c r="E11" s="16" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" ht="86.4" spans="1:6">
+    <row r="12" spans="1:6" ht="86.4">
       <c r="A12" s="15" t="s">
         <v>5</v>
       </c>
@@ -1695,7 +1145,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" ht="86.4" spans="1:6">
+    <row r="13" spans="1:6" ht="86.4">
       <c r="A13" s="15" t="s">
         <v>5</v>
       </c>
@@ -1710,26 +1160,41 @@
       </c>
       <c r="E13" s="16" t="s">
         <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="86.4">
+      <c r="A14" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.5555555555556" customWidth="1"/>
-    <col min="2" max="2" width="16.5555555555556" customWidth="1"/>
-    <col min="3" max="3" width="25.1111111111111" customWidth="1"/>
-    <col min="4" max="4" width="25.3333333333333" customWidth="1"/>
-    <col min="5" max="5" width="33.2222222222222" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="3" max="3" width="25.109375" customWidth="1"/>
+    <col min="4" max="4" width="25.33203125" customWidth="1"/>
+    <col min="5" max="5" width="33.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1749,7 +1214,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" ht="127.05" customHeight="1" spans="1:5">
+    <row r="2" spans="1:5" ht="127.05" customHeight="1">
       <c r="A2" s="5" t="s">
         <v>54</v>
       </c>
@@ -1766,7 +1231,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" ht="135" customHeight="1" spans="1:5">
+    <row r="3" spans="1:5" ht="135" customHeight="1">
       <c r="A3" s="5" t="s">
         <v>54</v>
       </c>
@@ -1783,7 +1248,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" ht="165" customHeight="1" spans="1:5">
+    <row r="4" spans="1:5" ht="165" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>54</v>
       </c>
@@ -1800,7 +1265,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" ht="129.6" spans="1:5">
+    <row r="5" spans="1:5" ht="144">
       <c r="A5" s="5" t="s">
         <v>54</v>
       </c>
@@ -1817,7 +1282,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" ht="144" spans="1:5">
+    <row r="6" spans="1:5" ht="144">
       <c r="A6" s="5" t="s">
         <v>54</v>
       </c>
@@ -1834,7 +1299,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" ht="115.2" spans="1:5">
+    <row r="7" spans="1:5" ht="144">
       <c r="A7" s="5" t="s">
         <v>54</v>
       </c>
@@ -1851,7 +1316,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="8" ht="115.2" spans="1:5">
+    <row r="8" spans="1:5" ht="115.2">
       <c r="A8" s="5" t="s">
         <v>54</v>
       </c>
@@ -1868,7 +1333,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" ht="86.4" spans="1:5">
+    <row r="9" spans="1:5" ht="100.8">
       <c r="A9" s="5" t="s">
         <v>54</v>
       </c>
@@ -1885,7 +1350,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="10" ht="100.8" spans="1:5">
+    <row r="10" spans="1:5" ht="100.8">
       <c r="A10" s="5" t="s">
         <v>54</v>
       </c>
@@ -1902,7 +1367,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" ht="100.8" spans="1:5">
+    <row r="11" spans="1:5" ht="100.8">
       <c r="A11" s="5" t="s">
         <v>54</v>
       </c>
@@ -1919,7 +1384,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="12" ht="156" customHeight="1" spans="1:5">
+    <row r="12" spans="1:5" ht="156" customHeight="1">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -1939,21 +1404,19 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.5555555555556" customWidth="1"/>
-    <col min="2" max="2" width="16.5555555555556" customWidth="1"/>
-    <col min="3" max="3" width="18.4444444444444" customWidth="1"/>
-    <col min="4" max="4" width="25.3333333333333" customWidth="1"/>
-    <col min="5" max="5" width="33.2222222222222" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="3" max="3" width="18.44140625" customWidth="1"/>
+    <col min="4" max="4" width="25.33203125" customWidth="1"/>
+    <col min="5" max="5" width="33.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1976,21 +1439,19 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.5555555555556" customWidth="1"/>
-    <col min="2" max="2" width="16.5555555555556" customWidth="1"/>
-    <col min="3" max="3" width="18.4444444444444" customWidth="1"/>
-    <col min="4" max="4" width="25.3333333333333" customWidth="1"/>
-    <col min="5" max="5" width="33.2222222222222" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="3" max="3" width="18.44140625" customWidth="1"/>
+    <col min="4" max="4" width="25.33203125" customWidth="1"/>
+    <col min="5" max="5" width="33.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2013,21 +1474,19 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.5555555555556" customWidth="1"/>
-    <col min="2" max="2" width="16.5555555555556" customWidth="1"/>
-    <col min="3" max="3" width="18.4444444444444" customWidth="1"/>
-    <col min="4" max="4" width="25.3333333333333" customWidth="1"/>
-    <col min="5" max="5" width="33.2222222222222" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="3" max="3" width="18.44140625" customWidth="1"/>
+    <col min="4" max="4" width="25.33203125" customWidth="1"/>
+    <col min="5" max="5" width="33.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2050,6 +1509,5 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added a new test case to LOGIN_FUNCTIONALITY as numericinput_to_password and testsheet.xlsx is updated
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="106">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -478,6 +478,21 @@
 2. enter the alphabet to the password variable.
 3. check that the entered data is entering in the password field.
 4. if entered then it is "PASSED: Alphabet keys work" otherwise "FAILED: Alphabet keys do not work". </t>
+  </si>
+  <si>
+    <t>TC_014</t>
+  </si>
+  <si>
+    <t>numericinput_to_password</t>
+  </si>
+  <si>
+    <t>To test the functionality of entering of the numeric values to the password field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
+2. enter the numeric value to the password variable.
+3. check that the entered data is entering in the password field.
+4. if entered then it is "PASSED: Number keys work" otherwise "FAILED: Number keys do not work". </t>
   </si>
 </sst>
 </file>
@@ -930,7 +945,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1177,6 +1192,23 @@
       </c>
       <c r="E14" s="19" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="86.4">
+      <c r="A15" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="D15" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="E15" s="19" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added a new test case named as specialsymbol_input_to_password to LOGIN_FUNCTIONALITY and updated the testsheet.xlsx with also updating the ChromeDriver to EdgeDriver to both specialsymbol_input_to_password and specialsymbol_input_to_username
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="110">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -493,6 +493,21 @@
 2. enter the numeric value to the password variable.
 3. check that the entered data is entering in the password field.
 4. if entered then it is "PASSED: Number keys work" otherwise "FAILED: Number keys do not work". </t>
+  </si>
+  <si>
+    <t>TC_015</t>
+  </si>
+  <si>
+    <t>specialsymbolinput_to_password</t>
+  </si>
+  <si>
+    <t>To test the functionality of entering of the special symbols to the password field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
+2. enter the symbol to the password variable.
+3. check that the entered data is entering in the password field.
+4. if entered then it is "TEST CASE PASS" otherwise "TEST CASE FAIL". </t>
   </si>
 </sst>
 </file>
@@ -945,7 +960,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1209,6 +1224,23 @@
       </c>
       <c r="E15" s="19" t="s">
         <v>105</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="86.4">
+      <c r="A16" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added a new test case name as spacesInputToUsername to LOGIN_FUNCTIONALITY and updated the testsheet.xlsx
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="114">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -508,6 +508,21 @@
 2. enter the symbol to the password variable.
 3. check that the entered data is entering in the password field.
 4. if entered then it is "TEST CASE PASS" otherwise "TEST CASE FAIL". </t>
+  </si>
+  <si>
+    <t>TC_016</t>
+  </si>
+  <si>
+    <t>spacesInputToUsername</t>
+  </si>
+  <si>
+    <t>To test the functionality of entering of the leading and trailing whitespaces to the username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
+2. enter the leading spacss name and trailing spaces.
+3. check that the entered data is entering in the username field.
+4. if entered then it is "PASS: Username field accepts leading and trailing spaces" otherwise "FAIL: Username field does not preserve the entered spaces". </t>
   </si>
 </sst>
 </file>
@@ -960,7 +975,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1241,6 +1256,23 @@
       </c>
       <c r="E16" s="19" t="s">
         <v>109</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="132.6" customHeight="1">
+      <c r="A17" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="E17" s="19" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added the new test case as passwordFieldMasking in LOGIN_FUNCTIONALITY and the respective update in the testsheet.slsx
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="118">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -524,17 +524,39 @@
 3. check that the entered data is entering in the username field.
 4. if entered then it is "PASS: Username field accepts leading and trailing spaces" otherwise "FAIL: Username field does not preserve the entered spaces". </t>
   </si>
+  <si>
+    <t>TC_017</t>
+  </si>
+  <si>
+    <t>passwordFieldMasking</t>
+  </si>
+  <si>
+    <t>To test the functionality of masking/hiding the password enter by the user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. open the url of the saucedemo webpage. 
+2. enter the password
+3. check that the type of the entered data is password..
+4. if match then it is "PASS: Password field masks the entered text" otherwise "FAIL: Password field is not masked". </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -565,6 +587,11 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="9">
@@ -628,24 +655,24 @@
   </borders>
   <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -661,32 +688,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -975,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1224,7 +1257,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="86.4">
+    <row r="15" spans="1:6" ht="122.4" customHeight="1">
       <c r="A15" s="15" t="s">
         <v>5</v>
       </c>
@@ -1241,7 +1274,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="86.4">
+    <row r="16" spans="1:6" ht="116.4" customHeight="1">
       <c r="A16" s="15" t="s">
         <v>5</v>
       </c>
@@ -1275,9 +1308,26 @@
         <v>113</v>
       </c>
     </row>
+    <row r="18" spans="1:5" ht="120" customHeight="1">
+      <c r="A18" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>117</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
added a new test case named as close_login_error_message in LOGIN_FUNCTIONALITY and testsheet.xlsx is updated
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="122">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -539,17 +539,40 @@
 3. check that the type of the entered data is password..
 4. if match then it is "PASS: Password field masks the entered text" otherwise "FAIL: Password field is not masked". </t>
   </si>
+  <si>
+    <t>TC_018</t>
+  </si>
+  <si>
+    <t>close_login_error_message</t>
+  </si>
+  <si>
+    <t>To test the functionality of closing the message that is displayed when the error shows.</t>
+  </si>
+  <si>
+    <t>1. open the url of the saucedemo webpage. 
+2. go to login button click on it without entering any username or password.
+3. check that the error message is displayed or not.
+4. if displayed then click on the "X" icon to close the error message that is displayed. 
+5. now check if the error message displayed then the test "FAILS" otherwise "PASS".</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -655,24 +678,24 @@
   </borders>
   <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -688,26 +711,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
@@ -716,8 +739,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1008,7 +1034,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1323,6 +1349,23 @@
       </c>
       <c r="E18" s="21" t="s">
         <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="163.80000000000001" customHeight="1">
+      <c r="A19" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added the new test case named as invalid_password_login in LOGIN_FUNCTIONALITY and testsheet.xlsx is updated
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="126">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -555,17 +555,39 @@
 4. if displayed then click on the "X" icon to close the error message that is displayed. 
 5. now check if the error message displayed then the test "FAILS" otherwise "PASS".</t>
   </si>
+  <si>
+    <t>TC_019</t>
+  </si>
+  <si>
+    <t>invalid_password_login</t>
+  </si>
+  <si>
+    <t>To test the functionality of login to the saucedemo by entering the invalid password.</t>
+  </si>
+  <si>
+    <t>1. open the url of the saucedemo webpage. 
+2. enter the username as standard_user.
+3. enter the wrong password.
+4. check the error if it matches then test case "PASSED" otherwise "FAILED" .</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -678,24 +700,24 @@
   </borders>
   <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -711,26 +733,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="11" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
@@ -739,8 +761,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1034,7 +1059,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1366,6 +1391,23 @@
       </c>
       <c r="E19" s="22" t="s">
         <v>121</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="72">
+      <c r="A20" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added a new test case named as invalid_username_valid_password in LOGIN_FUNCTIONALITY and testsheet.xlsx is updated till test case id TC_020
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="130">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -565,22 +565,46 @@
     <t>To test the functionality of login to the saucedemo by entering the invalid password.</t>
   </si>
   <si>
+    <t>TC_020</t>
+  </si>
+  <si>
+    <t>invalid_username_valid_password</t>
+  </si>
+  <si>
+    <t>To test the functionality of login to the saucedemo by entering the invalid username but the valid password.</t>
+  </si>
+  <si>
+    <t>1. open the url of the saucedemo webpage. 
+2. enter the username as invalid_user.
+3. enter the password as secret_sauce.
+4. click on the login button.
+5. check the error if it matches then test case "PASSED" otherwise "FAILED" .</t>
+  </si>
+  <si>
     <t>1. open the url of the saucedemo webpage. 
 2. enter the username as standard_user.
 3. enter the wrong password.
-4. check the error if it matches then test case "PASSED" otherwise "FAILED" .</t>
+4. click on the login button.
+5. check the error if it matches then test case "PASSED" otherwise "FAILED" .</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -700,24 +724,24 @@
   </borders>
   <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -733,26 +757,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="11" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="11" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="11" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="11" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
@@ -761,8 +785,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1059,7 +1086,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1393,7 +1420,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="72">
+    <row r="20" spans="1:5" ht="111" customHeight="1">
       <c r="A20" s="18" t="s">
         <v>5</v>
       </c>
@@ -1406,8 +1433,25 @@
       <c r="D20" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="E20" s="23" t="s">
+      <c r="E20" s="24" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="111" customHeight="1">
+      <c r="A21" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="13" t="s">
         <v>125</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="D21" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="E21" s="24" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added a new test case named as caseSensitiveUsernameTest in LOGIN_FUNCTIONALITY and testsheet.xlsx is updated till tc_021
</commit_message>
<xml_diff>
--- a/testsheet.xlsx
+++ b/testsheet.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="134">
   <si>
     <t>FUNCTIONALITY</t>
   </si>
@@ -587,17 +587,40 @@
 4. click on the login button.
 5. check the error if it matches then test case "PASSED" otherwise "FAILED" .</t>
   </si>
+  <si>
+    <t>TC_021</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> caseSensitiveUsernameTest</t>
+  </si>
+  <si>
+    <t>To test the functionality of casesensitive login to the saucedemo by entering the username in caps lock .</t>
+  </si>
+  <si>
+    <t>1. open the url of the saucedemo webpage. 
+2. enter the username as STANDARD_USER(upper case).
+3. enter the password as secret_sauce.
+4. click on the login button.
+5. check the error if it matches then test case "PASS AND USERNAME IS CASE-SENSITIVE" and if login done also using the uppercase of the Username then "FAIL Unexpected login result." .</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -724,24 +747,24 @@
   </borders>
   <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -757,26 +780,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="11" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="11" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="11" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="11" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="11" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
@@ -785,8 +808,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1086,7 +1112,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1452,6 +1478,23 @@
       </c>
       <c r="E21" s="24" t="s">
         <v>128</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="129.6">
+      <c r="A22" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E22" s="25" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>